<commit_message>
Fruit Master v1.1: pay the highest win, rebalance directly, validate by CI
- Evaluation now pays the highest qualifying win. In v1.0 the fixed check
  order made W W C pay 4 and W W L pay 8 while W W blank paid 10 (27 of
  8,000 outcomes). A test checks that adding a symbol never lowers the win.
- Rebalanced: RTP is linear in each pay, so the 2 Wilds pay for 96% is
  solved directly (6.05) and rounded to 6. RTP 95.9875%, hit frequency
  22.6125%, sigma 3.8142.
- Simulation validated with 95% confidence intervals instead of a fixed
  1 pp rule; vectorised with numpy default_rng.
- Shared model module, PAR-style table, volatility index, tests,
  requirements.txt; docs and Excel workbooks updated.
</commit_message>
<xml_diff>
--- a/excel/Fruit_Master.xlsx
+++ b/excel/Fruit_Master.xlsx
@@ -1044,11 +1044,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CCC with Wild</t>
+          <t>CCC with Wild (not 2 Wilds)</t>
         </is>
       </c>
       <c r="B6">
-        <f>(ReelStrips!$F2 + ReelStrips!$F6) * (ReelStrips!$G2 + ReelStrips!$G6)  * (ReelStrips!$H2 + ReelStrips!$H6) - 1</f>
+        <f>(ReelStrips!$F2 + ReelStrips!$F6) * (ReelStrips!$G2 + ReelStrips!$G6) * (ReelStrips!$H2 + ReelStrips!$H6) - 1 - (ReelStrips!$F6*ReelStrips!$G6*ReelStrips!$H2 + ReelStrips!$F6*ReelStrips!$G2*ReelStrips!$H6 + ReelStrips!$F2*ReelStrips!$G6*ReelStrips!$H6)</f>
         <v/>
       </c>
       <c r="C6">
@@ -1067,11 +1067,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Exactly 2 Wilds</t>
+          <t>Exactly 2 Wilds (third C or blank)</t>
         </is>
       </c>
       <c r="B7">
-        <f>(ReelStrips!$F6*ReelStrips!$G6*ReelStrips!$H7)+(ReelStrips!$F6*ReelStrips!$G7*ReelStrips!$H6)+(ReelStrips!$F7*ReelStrips!$G6*ReelStrips!$H6)</f>
+        <f>ReelStrips!$F6*ReelStrips!$G6*(ReelStrips!$H2+ReelStrips!$H7) + ReelStrips!$F6*(ReelStrips!$G2+ReelStrips!$G7)*ReelStrips!$H6 + (ReelStrips!$F2+ReelStrips!$F7)*ReelStrips!$G6*ReelStrips!$H6</f>
         <v/>
       </c>
       <c r="C7">
@@ -1145,21 +1145,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Note: Ways for 'Exactly 1 Wild' and 'CC any' involve multi-case exclusion logic</t>
+          <t>Highest win is paid: W W C pays 2 Wilds (6) rather than CCC (4); W W L, W W O, W W B pay their triple (8 or more).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>that is impractical as a single Excel formula; values cross-validated via full</t>
+          <t>Ways for 'Exactly 1 Wild' and 'CC any' involve multi-case exclusions that are impractical as one formula;</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>enumeration in src/enumerate_rtp.py (category breakdown of all 8,000 outcomes).</t>
+          <t>those counts come from the full enumeration in src/enumerate_rtp.py (all 8,000 outcomes).</t>
         </is>
       </c>
     </row>
@@ -1174,7 +1174,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="17.77734375" customWidth="1" min="1" max="1"/>
@@ -1238,7 +1238,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -1269,6 +1269,13 @@
       </c>
       <c r="B9" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Evaluation: every qualifying combination is found and only the highest pay is awarded (v1.1).</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1282,7 +1289,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="35.77734375" customWidth="1" min="1" max="1"/>
@@ -1308,7 +1315,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="3">
@@ -1370,7 +1377,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>46239</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="9">
@@ -1388,7 +1395,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.961125</v>
+        <v>0.959875</v>
       </c>
     </row>
     <row r="11">
@@ -1398,7 +1405,7 @@
         </is>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.961125</v>
+        <v>0.959875</v>
       </c>
     </row>
     <row r="12">
@@ -1440,7 +1447,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Full eunmeration of 8000 outcomes</t>
+          <t>Full enumeration of 8,000 outcomes</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1465,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.966397</v>
+        <v>0.960006</v>
       </c>
     </row>
     <row r="18">
@@ -1468,7 +1475,7 @@
         </is>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.966397</v>
+        <v>0.960006</v>
       </c>
     </row>
     <row r="19">
@@ -1478,7 +1485,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.5272</v>
+        <v>0.0131</v>
       </c>
     </row>
     <row r="20">
@@ -1488,7 +1495,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>3.82237</v>
+        <v>3.8049</v>
       </c>
     </row>
     <row r="21">
@@ -1498,7 +1505,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.226385</v>
+        <v>0.22634</v>
       </c>
     </row>
     <row r="22">
@@ -1508,7 +1515,7 @@
         </is>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.226385</v>
+        <v>0.22634</v>
       </c>
     </row>
     <row r="23">
@@ -1556,7 +1563,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Complete – balanced &amp; validated</t>
+          <t>Complete – v1.1: highest-win rule, rebalanced, validated by 95% CI</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1575,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Initial 132.3% → final 96.11%</t>
+          <t>132.3% → 96.11% (v1.0) → 97.44% after rule fix → 95.99% (2 Wilds solved, rounded to 6)</t>
         </is>
       </c>
     </row>
@@ -1580,7 +1587,39 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>enumerate_rtp.py, simulation.py, game_math_document.md</t>
+          <t>slot_model.py, enumerate_rtp.py, simulation.py, game_math_document.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Std deviation (exact)</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>3.8142</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Volatility index (90%)</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>6.27</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Simulation 95% CI</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>95.2548% – 96.7464% (theory inside)</t>
         </is>
       </c>
     </row>

</xml_diff>